<commit_message>
Week 6 Day 2 Uploads
</commit_message>
<xml_diff>
--- a/Shapiro 2025 Project/Python SquidPy/summary_matrix_6_27.xlsx
+++ b/Shapiro 2025 Project/Python SquidPy/summary_matrix_6_27.xlsx
@@ -8,19 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ejohns\Documents\GitHub\2025-Dinh-Lab-Research-Project\Shapiro 2025 Project\Python SquidPy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55707241-21BB-463A-A555-FA9FEB35084A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB5A3982-1730-4DEC-B8E0-9F3FE6E58093}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-210" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$O$67</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="92">
   <si>
     <t>Sample ID</t>
   </si>
@@ -269,6 +285,33 @@
   </si>
   <si>
     <t>c_3_20_</t>
+  </si>
+  <si>
+    <t>Average Distance to all Cells (µm)</t>
+  </si>
+  <si>
+    <t>CD4</t>
+  </si>
+  <si>
+    <t>CD8</t>
+  </si>
+  <si>
+    <t>Treg</t>
+  </si>
+  <si>
+    <t>Tumor</t>
+  </si>
+  <si>
+    <t>Average R</t>
+  </si>
+  <si>
+    <t>Average NR</t>
+  </si>
+  <si>
+    <t>Average Distance to Closest Cell (µm)</t>
+  </si>
+  <si>
+    <t>Average Paired Distance (µm)</t>
   </si>
 </sst>
 </file>
@@ -297,7 +340,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -320,15 +363,104 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -631,9 +763,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O67"/>
+  <dimension ref="A1:Z67"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="3" max="3" width="16.90625" customWidth="1"/>
+    <col min="4" max="5" width="23.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25.7265625" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="15.54296875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15.90625" bestFit="1" customWidth="1"/>
@@ -641,9 +777,14 @@
     <col min="12" max="13" width="17.7265625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="18.08984375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="19.90625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="32" bestFit="1" customWidth="1"/>
+    <col min="18" max="20" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.54296875" customWidth="1"/>
+    <col min="24" max="24" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="17.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -689,8 +830,14 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="X1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -736,8 +883,25 @@
       <c r="O2">
         <v>16.29900190481662</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q2" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="R2" s="3"/>
+      <c r="S2" s="3"/>
+      <c r="T2" s="3"/>
+      <c r="U2" s="4"/>
+      <c r="X2">
+        <v>273.97261431482508</v>
+      </c>
+      <c r="Y2">
+        <v>436.8167220452529</v>
+      </c>
+      <c r="Z2">
+        <f>IF(X2&gt;Y2,1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -783,8 +947,31 @@
       <c r="O3">
         <v>11.824233477580639</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q3" s="5"/>
+      <c r="R3" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="S3" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="T3" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="U3" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="X3">
+        <v>28.753049449632279</v>
+      </c>
+      <c r="Y3">
+        <v>44.325139628945337</v>
+      </c>
+      <c r="Z3">
+        <f t="shared" ref="Z3:Z66" si="0">IF(X3&gt;Y3,1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -830,8 +1017,37 @@
       <c r="O4">
         <v>28.402609109711591</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q4" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="R4" s="10">
+        <f>AVERAGE(H2:H34)</f>
+        <v>372.02843052333685</v>
+      </c>
+      <c r="S4" s="10">
+        <f t="shared" ref="S4:U4" si="1">AVERAGE(I2:I34)</f>
+        <v>395.97629222169343</v>
+      </c>
+      <c r="T4" s="10">
+        <f t="shared" si="1"/>
+        <v>370.63275544116249</v>
+      </c>
+      <c r="U4" s="6">
+        <f t="shared" si="1"/>
+        <v>390.79140061353661</v>
+      </c>
+      <c r="X4">
+        <v>52.528239826469722</v>
+      </c>
+      <c r="Y4">
+        <v>54.468324370900667</v>
+      </c>
+      <c r="Z4">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -877,8 +1093,37 @@
       <c r="O5">
         <v>17.1375220176573</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q5" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="R5" s="8">
+        <f>AVERAGE(H35:H67)</f>
+        <v>397.17706282568031</v>
+      </c>
+      <c r="S5" s="8">
+        <f t="shared" ref="S5:U5" si="2">AVERAGE(I35:I67)</f>
+        <v>396.66106433973192</v>
+      </c>
+      <c r="T5" s="8">
+        <f t="shared" si="2"/>
+        <v>390.84053072994607</v>
+      </c>
+      <c r="U5" s="9">
+        <f t="shared" si="2"/>
+        <v>412.3701709221603</v>
+      </c>
+      <c r="X5">
+        <v>86.062534523483833</v>
+      </c>
+      <c r="Y5">
+        <v>114.1410885124926</v>
+      </c>
+      <c r="Z5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -924,2452 +1169,3077 @@
       <c r="O6">
         <v>50.561472939676747</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="X6">
+        <v>19.640477871993308</v>
+      </c>
+      <c r="Y6">
+        <v>11.740741964573219</v>
+      </c>
+      <c r="Z6">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B7">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D7">
-        <v>95.952061780353603</v>
+        <v>59.507652420430787</v>
       </c>
       <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <v>191.8574369369565</v>
+        <v>94.427574560927127</v>
       </c>
       <c r="G7">
-        <v>10.28284606445969</v>
+        <v>27.41631011367506</v>
       </c>
       <c r="H7">
-        <v>482.95669182112181</v>
+        <v>371.65706003860458</v>
       </c>
       <c r="I7">
-        <v>0</v>
-      </c>
-      <c r="J7">
-        <v>362.76347828603468</v>
+        <v>337.34162297852117</v>
       </c>
       <c r="K7">
-        <v>446.3343062424355</v>
+        <v>409.85504318097742</v>
       </c>
       <c r="L7">
-        <v>289.24872066023192</v>
+        <v>77.912690278094317</v>
       </c>
       <c r="M7">
-        <v>0</v>
-      </c>
-      <c r="N7">
-        <v>214.6767046368949</v>
+        <v>109.9101454208396</v>
       </c>
       <c r="O7">
-        <v>10.28284606445969</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+        <v>28.954481905811559</v>
+      </c>
+      <c r="X7">
+        <v>59.507652420430787</v>
+      </c>
+      <c r="Y7">
+        <v>77.912690278094317</v>
+      </c>
+      <c r="Z7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B8">
-        <v>29</v>
+        <v>118</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D8">
-        <v>91.71700113373214</v>
+        <v>51.302748247358238</v>
       </c>
       <c r="E8">
-        <v>50.58835564570748</v>
+        <v>74.764000416197007</v>
       </c>
       <c r="F8">
-        <v>573.29576775519558</v>
+        <v>72.36446002053934</v>
       </c>
       <c r="G8">
-        <v>79.245818219534939</v>
+        <v>18.98864602292992</v>
       </c>
       <c r="H8">
-        <v>403.76236488191728</v>
+        <v>373.40345026243239</v>
       </c>
       <c r="I8">
-        <v>465.33915893749509</v>
+        <v>392.53826665263227</v>
       </c>
       <c r="J8">
-        <v>573.29576775519558</v>
+        <v>363.70192158073212</v>
       </c>
       <c r="K8">
-        <v>370.05124866902253</v>
+        <v>372.31706008587622</v>
       </c>
       <c r="L8">
-        <v>177.05480894775809</v>
+        <v>75.959703399638286</v>
       </c>
       <c r="M8">
-        <v>103.8138812333322</v>
+        <v>125.8716450099641</v>
       </c>
       <c r="N8">
-        <v>15.864217850243991</v>
+        <v>110.5666114232605</v>
       </c>
       <c r="O8">
-        <v>104.282643969308</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+        <v>21.019737477870681</v>
+      </c>
+      <c r="X8">
+        <v>51.302748247358238</v>
+      </c>
+      <c r="Y8">
+        <v>75.959703399638286</v>
+      </c>
+      <c r="Z8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B9">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D9">
-        <v>127.0414892215851</v>
+        <v>33.266268562351023</v>
       </c>
       <c r="E9">
-        <v>161.79046065770581</v>
+        <v>55.60825060785254</v>
       </c>
       <c r="F9">
-        <v>193.4390885246533</v>
+        <v>56.348116386193098</v>
       </c>
       <c r="G9">
-        <v>16.599355594149358</v>
+        <v>17.132383663955629</v>
       </c>
       <c r="H9">
-        <v>444.57000559024959</v>
+        <v>372.21839935632988</v>
       </c>
       <c r="I9">
-        <v>469.29795805113702</v>
+        <v>360.13145236715178</v>
       </c>
       <c r="J9">
-        <v>477.60802690206509</v>
+        <v>359.95717735800213</v>
       </c>
       <c r="K9">
-        <v>396.91837570010819</v>
+        <v>355.32793612225208</v>
       </c>
       <c r="L9">
-        <v>234.37095667492471</v>
+        <v>67.048185061591653</v>
       </c>
       <c r="M9">
-        <v>263.16988534515559</v>
+        <v>82.278561233989166</v>
       </c>
       <c r="N9">
-        <v>264.95906826024179</v>
+        <v>107.362634770817</v>
       </c>
       <c r="O9">
-        <v>19.25326026909352</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+        <v>18.80299297831251</v>
+      </c>
+      <c r="Q9" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="R9" s="3"/>
+      <c r="S9" s="3"/>
+      <c r="T9" s="3"/>
+      <c r="U9" s="4"/>
+      <c r="X9">
+        <v>33.266268562351023</v>
+      </c>
+      <c r="Y9">
+        <v>67.048185061591653</v>
+      </c>
+      <c r="Z9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B10">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
         <v>16</v>
       </c>
       <c r="D10">
-        <v>59.507652420430787</v>
+        <v>154.12164705344779</v>
       </c>
       <c r="E10">
-        <v>94.427574560927127</v>
+        <v>170.1422961963998</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>142.6864087910603</v>
       </c>
       <c r="G10">
-        <v>27.41631011367506</v>
+        <v>15.410779320906549</v>
       </c>
       <c r="H10">
-        <v>371.65706003860458</v>
+        <v>449.8256929072935</v>
       </c>
       <c r="I10">
-        <v>337.34162297852117</v>
+        <v>457.58429450624982</v>
       </c>
       <c r="J10">
-        <v>0</v>
+        <v>401.80596361963222</v>
       </c>
       <c r="K10">
-        <v>409.85504318097742</v>
+        <v>446.21566005514683</v>
       </c>
       <c r="L10">
-        <v>77.912690278094317</v>
+        <v>248.8254906734555</v>
       </c>
       <c r="M10">
-        <v>109.9101454208396</v>
+        <v>316.308846953292</v>
       </c>
       <c r="N10">
-        <v>0</v>
+        <v>255.16000173033439</v>
       </c>
       <c r="O10">
-        <v>28.954481905811559</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+        <v>18.28001688760347</v>
+      </c>
+      <c r="Q10" s="5"/>
+      <c r="R10" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="S10" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="T10" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="U10" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="X10">
+        <v>154.12164705344779</v>
+      </c>
+      <c r="Y10">
+        <v>248.8254906734555</v>
+      </c>
+      <c r="Z10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B11">
-        <v>118</v>
+        <v>7</v>
       </c>
       <c r="C11" t="s">
         <v>16</v>
       </c>
       <c r="D11">
-        <v>51.302748247358238</v>
+        <v>39.116455608961068</v>
       </c>
       <c r="E11">
-        <v>74.764000416197007</v>
+        <v>103.59108581784071</v>
       </c>
       <c r="F11">
-        <v>72.36446002053934</v>
+        <v>107.05660549423411</v>
       </c>
       <c r="G11">
-        <v>18.98864602292992</v>
+        <v>40.047720266079089</v>
       </c>
       <c r="H11">
-        <v>373.40345026243239</v>
+        <v>276.43714232757418</v>
       </c>
       <c r="I11">
-        <v>392.53826665263227</v>
+        <v>281.2925659253541</v>
       </c>
       <c r="J11">
-        <v>363.70192158073212</v>
+        <v>226.33081449373759</v>
       </c>
       <c r="K11">
-        <v>372.31706008587622</v>
+        <v>365.36439885079272</v>
       </c>
       <c r="L11">
-        <v>75.959703399638286</v>
+        <v>39.19774774745057</v>
       </c>
       <c r="M11">
-        <v>125.8716450099641</v>
+        <v>125.28449579132889</v>
       </c>
       <c r="N11">
-        <v>110.5666114232605</v>
+        <v>111.82314130661661</v>
       </c>
       <c r="O11">
-        <v>21.019737477870681</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+        <v>45.269028367780898</v>
+      </c>
+      <c r="Q11" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="R11" s="10">
+        <f>AVERAGE(D2:D34)</f>
+        <v>67.744588763797367</v>
+      </c>
+      <c r="S11" s="10">
+        <f t="shared" ref="S11:U11" si="3">AVERAGE(E2:E34)</f>
+        <v>115.53116313522285</v>
+      </c>
+      <c r="T11" s="10">
+        <f t="shared" si="3"/>
+        <v>116.59405449592236</v>
+      </c>
+      <c r="U11" s="6">
+        <f t="shared" si="3"/>
+        <v>23.667671849531569</v>
+      </c>
+      <c r="X11">
+        <v>39.116455608961068</v>
+      </c>
+      <c r="Y11">
+        <v>39.19774774745057</v>
+      </c>
+      <c r="Z11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B12">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="C12" t="s">
         <v>16</v>
       </c>
       <c r="D12">
-        <v>33.266268562351023</v>
+        <v>86.823432187811136</v>
       </c>
       <c r="E12">
-        <v>55.60825060785254</v>
+        <v>137.5525511065108</v>
       </c>
       <c r="F12">
-        <v>56.348116386193098</v>
+        <v>148.8184777874595</v>
       </c>
       <c r="G12">
-        <v>17.132383663955629</v>
+        <v>27.957135595425299</v>
       </c>
       <c r="H12">
-        <v>372.21839935632988</v>
+        <v>416.84824177243252</v>
       </c>
       <c r="I12">
-        <v>360.13145236715178</v>
+        <v>449.50279347255628</v>
       </c>
       <c r="J12">
-        <v>359.95717735800213</v>
+        <v>422.72586749450801</v>
       </c>
       <c r="K12">
-        <v>355.32793612225208</v>
+        <v>400.10234501837192</v>
       </c>
       <c r="L12">
-        <v>67.048185061591653</v>
+        <v>120.92291156738079</v>
       </c>
       <c r="M12">
-        <v>82.278561233989166</v>
+        <v>264.29524124143478</v>
       </c>
       <c r="N12">
-        <v>107.362634770817</v>
+        <v>247.22641867896701</v>
       </c>
       <c r="O12">
-        <v>18.80299297831251</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+        <v>28.660485183357562</v>
+      </c>
+      <c r="Q12" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="R12" s="8">
+        <f>AVERAGE(D35:D67)</f>
+        <v>73.731341932425181</v>
+      </c>
+      <c r="S12" s="8">
+        <f t="shared" ref="S12:U12" si="4">AVERAGE(E35:E67)</f>
+        <v>117.48695217896316</v>
+      </c>
+      <c r="T12" s="8">
+        <f t="shared" si="4"/>
+        <v>126.10667659519702</v>
+      </c>
+      <c r="U12" s="9">
+        <f t="shared" si="4"/>
+        <v>25.317063123266859</v>
+      </c>
+      <c r="X12">
+        <v>86.823432187811136</v>
+      </c>
+      <c r="Y12">
+        <v>120.92291156738079</v>
+      </c>
+      <c r="Z12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B13">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C13" t="s">
         <v>16</v>
       </c>
       <c r="D13">
-        <v>154.12164705344779</v>
+        <v>30.766121934381921</v>
       </c>
       <c r="E13">
-        <v>170.1422961963998</v>
+        <v>44.039743682502163</v>
       </c>
       <c r="F13">
-        <v>142.6864087910603</v>
+        <v>36.581881447312469</v>
       </c>
       <c r="G13">
-        <v>15.410779320906549</v>
+        <v>24.721430963236589</v>
       </c>
       <c r="H13">
-        <v>449.8256929072935</v>
+        <v>413.14862247489589</v>
       </c>
       <c r="I13">
-        <v>457.58429450624982</v>
+        <v>451.10349983725553</v>
       </c>
       <c r="J13">
-        <v>401.80596361963222</v>
+        <v>410.40369496310711</v>
       </c>
       <c r="K13">
-        <v>446.21566005514683</v>
+        <v>406.69990135419482</v>
       </c>
       <c r="L13">
-        <v>248.8254906734555</v>
+        <v>40.699985976653792</v>
       </c>
       <c r="M13">
-        <v>316.308846953292</v>
+        <v>45.977199011883798</v>
       </c>
       <c r="N13">
-        <v>255.16000173033439</v>
+        <v>53.984083403920202</v>
       </c>
       <c r="O13">
-        <v>18.28001688760347</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+        <v>25.16810827451943</v>
+      </c>
+      <c r="X13">
+        <v>30.766121934381921</v>
+      </c>
+      <c r="Y13">
+        <v>40.699985976653792</v>
+      </c>
+      <c r="Z13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="B14">
-        <v>7</v>
+        <v>80</v>
       </c>
       <c r="C14" t="s">
         <v>16</v>
       </c>
       <c r="D14">
-        <v>39.116455608961068</v>
+        <v>198.09500092572199</v>
       </c>
       <c r="E14">
-        <v>103.59108581784071</v>
+        <v>209.00454740982869</v>
       </c>
       <c r="F14">
-        <v>107.05660549423411</v>
+        <v>337.02747504390419</v>
       </c>
       <c r="G14">
-        <v>40.047720266079089</v>
+        <v>15.22752458646492</v>
       </c>
       <c r="H14">
-        <v>276.43714232757418</v>
+        <v>505.76201768521298</v>
       </c>
       <c r="I14">
-        <v>281.2925659253541</v>
+        <v>565.83396146383166</v>
       </c>
       <c r="J14">
-        <v>226.33081449373759</v>
+        <v>497.28619293931843</v>
       </c>
       <c r="K14">
-        <v>365.36439885079272</v>
+        <v>368.68422318270018</v>
       </c>
       <c r="L14">
-        <v>39.19774774745057</v>
+        <v>401.10201604492812</v>
       </c>
       <c r="M14">
-        <v>125.28449579132889</v>
+        <v>247.6232090369173</v>
       </c>
       <c r="N14">
-        <v>111.82314130661661</v>
+        <v>307.26348235991912</v>
       </c>
       <c r="O14">
-        <v>45.269028367780898</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+        <v>19.02130589960159</v>
+      </c>
+      <c r="X14">
+        <v>198.09500092572199</v>
+      </c>
+      <c r="Y14">
+        <v>401.10201604492812</v>
+      </c>
+      <c r="Z14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B15">
-        <v>19</v>
+        <v>495</v>
       </c>
       <c r="C15" t="s">
         <v>16</v>
       </c>
       <c r="D15">
-        <v>86.823432187811136</v>
+        <v>38.858369836070679</v>
       </c>
       <c r="E15">
-        <v>137.5525511065108</v>
+        <v>23.003241880869538</v>
       </c>
       <c r="F15">
-        <v>148.8184777874595</v>
+        <v>55.529786383888649</v>
       </c>
       <c r="G15">
-        <v>27.957135595425299</v>
+        <v>29.69081823332094</v>
       </c>
       <c r="H15">
-        <v>416.84824177243252</v>
+        <v>373.3529496894771</v>
       </c>
       <c r="I15">
-        <v>449.50279347255628</v>
+        <v>372.97320959068219</v>
       </c>
       <c r="J15">
-        <v>422.72586749450801</v>
+        <v>380.82651312061648</v>
       </c>
       <c r="K15">
-        <v>400.10234501837192</v>
+        <v>399.01944703871101</v>
       </c>
       <c r="L15">
-        <v>120.92291156738079</v>
+        <v>42.167018507148647</v>
       </c>
       <c r="M15">
-        <v>264.29524124143478</v>
+        <v>47.935403518265773</v>
       </c>
       <c r="N15">
-        <v>247.22641867896701</v>
+        <v>28.939664094241479</v>
       </c>
       <c r="O15">
-        <v>28.660485183357562</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+        <v>90.152138198962177</v>
+      </c>
+      <c r="Q15" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="R15" s="3"/>
+      <c r="S15" s="3"/>
+      <c r="T15" s="3"/>
+      <c r="U15" s="4"/>
+      <c r="X15">
+        <v>38.858369836070679</v>
+      </c>
+      <c r="Y15">
+        <v>42.167018507148647</v>
+      </c>
+      <c r="Z15">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B16">
-        <v>33</v>
+        <v>147</v>
       </c>
       <c r="C16" t="s">
         <v>16</v>
       </c>
       <c r="D16">
-        <v>30.766121934381921</v>
+        <v>157.75639828891099</v>
       </c>
       <c r="E16">
-        <v>44.039743682502163</v>
+        <v>209.50239690610761</v>
       </c>
       <c r="F16">
-        <v>36.581881447312469</v>
+        <v>129.9183484252321</v>
       </c>
       <c r="G16">
-        <v>24.721430963236589</v>
+        <v>15.466662288797361</v>
       </c>
       <c r="H16">
-        <v>413.14862247489589</v>
+        <v>399.38009470532103</v>
       </c>
       <c r="I16">
-        <v>451.10349983725553</v>
+        <v>394.69514364353279</v>
       </c>
       <c r="J16">
-        <v>410.40369496310711</v>
+        <v>379.86227938982069</v>
       </c>
       <c r="K16">
-        <v>406.69990135419482</v>
+        <v>347.22455284469203</v>
       </c>
       <c r="L16">
-        <v>40.699985976653792</v>
+        <v>216.89246388962491</v>
       </c>
       <c r="M16">
-        <v>45.977199011883798</v>
+        <v>87.143027401900639</v>
       </c>
       <c r="N16">
-        <v>53.984083403920202</v>
+        <v>163.42557540023401</v>
       </c>
       <c r="O16">
-        <v>25.16810827451943</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
+        <v>27.679016770206019</v>
+      </c>
+      <c r="Q16" s="5"/>
+      <c r="R16" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="S16" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="T16" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="U16" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="X16">
+        <v>157.75639828891099</v>
+      </c>
+      <c r="Y16">
+        <v>216.89246388962491</v>
+      </c>
+      <c r="Z16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="B17">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C17" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D17">
-        <v>56.611725681597093</v>
+        <v>26.514968970004919</v>
       </c>
       <c r="E17">
-        <v>139.1030672878758</v>
+        <v>27.930890454349871</v>
       </c>
       <c r="F17">
-        <v>91.895401500037494</v>
+        <v>42.841332240449987</v>
       </c>
       <c r="G17">
-        <v>24.01054211217313</v>
+        <v>27.092258521692589</v>
       </c>
       <c r="H17">
-        <v>406.31802223501558</v>
+        <v>401.24140347035029</v>
       </c>
       <c r="I17">
-        <v>461.4504742414772</v>
+        <v>390.58785075394218</v>
       </c>
       <c r="J17">
-        <v>423.70214873900591</v>
+        <v>385.15892322945092</v>
       </c>
       <c r="K17">
-        <v>396.58512384641921</v>
+        <v>376.91842529035341</v>
       </c>
       <c r="L17">
-        <v>82.57993141699049</v>
+        <v>29.380245318894701</v>
       </c>
       <c r="M17">
-        <v>289.25155042577393</v>
+        <v>29.05871847571445</v>
       </c>
       <c r="N17">
-        <v>240.02224576808149</v>
+        <v>44.779463616152093</v>
       </c>
       <c r="O17">
-        <v>32.060364125303259</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
+        <v>28.10572963842079</v>
+      </c>
+      <c r="Q17" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="R17" s="10">
+        <f>AVERAGE(L2:L34)</f>
+        <v>106.37717841294388</v>
+      </c>
+      <c r="S17" s="10">
+        <f t="shared" ref="S17:U17" si="5">AVERAGE(M2:M34)</f>
+        <v>143.37377591445738</v>
+      </c>
+      <c r="T17" s="10">
+        <f t="shared" si="5"/>
+        <v>135.18479339175775</v>
+      </c>
+      <c r="U17" s="6">
+        <f t="shared" si="5"/>
+        <v>33.42196973050283</v>
+      </c>
+      <c r="X17">
+        <v>26.514968970004919</v>
+      </c>
+      <c r="Y17">
+        <v>29.380245318894701</v>
+      </c>
+      <c r="Z17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="B18">
-        <v>458</v>
+        <v>100</v>
       </c>
       <c r="C18" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D18">
-        <v>65.001757273467902</v>
+        <v>24.227225068400369</v>
       </c>
       <c r="E18">
-        <v>43.860218685961733</v>
+        <v>35.480122730762197</v>
       </c>
       <c r="F18">
-        <v>92.983017447037724</v>
+        <v>37.736667367152322</v>
       </c>
       <c r="G18">
-        <v>17.231497919734071</v>
+        <v>21.86016814579628</v>
       </c>
       <c r="H18">
-        <v>345.52684228687423</v>
+        <v>353.42302267168043</v>
       </c>
       <c r="I18">
-        <v>340.95971503899079</v>
+        <v>357.69953615911032</v>
       </c>
       <c r="J18">
-        <v>349.27117327367802</v>
+        <v>341.00883908011042</v>
       </c>
       <c r="K18">
-        <v>408.81734039456319</v>
+        <v>360.39677598267832</v>
       </c>
       <c r="L18">
-        <v>36.55900717081883</v>
+        <v>29.87344806809881</v>
       </c>
       <c r="M18">
-        <v>32.989309807573413</v>
+        <v>44.057606804907749</v>
       </c>
       <c r="N18">
-        <v>25.83869576242795</v>
+        <v>55.444262774132113</v>
       </c>
       <c r="O18">
-        <v>27.028190687332021</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+        <v>23.691980427160729</v>
+      </c>
+      <c r="Q18" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="R18" s="8">
+        <f>AVERAGE(L35:L67)</f>
+        <v>125.44200025955956</v>
+      </c>
+      <c r="S18" s="8">
+        <f t="shared" ref="S18:U18" si="6">AVERAGE(M35:M67)</f>
+        <v>131.94632045329612</v>
+      </c>
+      <c r="T18" s="8">
+        <f t="shared" si="6"/>
+        <v>122.33906652494956</v>
+      </c>
+      <c r="U18" s="9">
+        <f t="shared" si="6"/>
+        <v>31.868305920625687</v>
+      </c>
+      <c r="X18">
+        <v>24.227225068400369</v>
+      </c>
+      <c r="Y18">
+        <v>29.87344806809881</v>
+      </c>
+      <c r="Z18">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:26" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="B19">
-        <v>416</v>
+        <v>48</v>
       </c>
       <c r="C19" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D19">
-        <v>83.028796498862903</v>
+        <v>26.98944663668691</v>
       </c>
       <c r="E19">
-        <v>71.287098259342031</v>
+        <v>33.895915994301347</v>
       </c>
       <c r="F19">
-        <v>130.9636023752484</v>
+        <v>37.256565678364083</v>
       </c>
       <c r="G19">
-        <v>15.836556562469269</v>
+        <v>11.128145913861321</v>
       </c>
       <c r="H19">
-        <v>398.04948882641889</v>
+        <v>312.23451990534687</v>
       </c>
       <c r="I19">
-        <v>393.38916107738578</v>
+        <v>355.43723262233408</v>
       </c>
       <c r="J19">
-        <v>401.22822159322033</v>
+        <v>308.78392064557579</v>
       </c>
       <c r="K19">
-        <v>368.02768399560898</v>
+        <v>333.21999986488811</v>
       </c>
       <c r="L19">
-        <v>59.702356290752988</v>
+        <v>37.71408536963763</v>
       </c>
       <c r="M19">
-        <v>51.002124872064037</v>
+        <v>92.632080716457835</v>
       </c>
       <c r="N19">
-        <v>64.609602756275436</v>
+        <v>79.273890310224957</v>
       </c>
       <c r="O19">
-        <v>20.955192969868751</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
+        <v>11.31663605866877</v>
+      </c>
+      <c r="X19">
+        <v>26.98944663668691</v>
+      </c>
+      <c r="Y19">
+        <v>37.71408536963763</v>
+      </c>
+      <c r="Z19">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="B20">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C20" t="s">
         <v>16</v>
       </c>
       <c r="D20">
-        <v>198.09500092572199</v>
+        <v>60.699558981672652</v>
       </c>
       <c r="E20">
-        <v>209.00454740982869</v>
+        <v>31.472697816142691</v>
       </c>
       <c r="F20">
-        <v>337.02747504390419</v>
+        <v>208.58516339246131</v>
       </c>
       <c r="G20">
-        <v>15.22752458646492</v>
+        <v>26.271065972465401</v>
       </c>
       <c r="H20">
-        <v>505.76201768521298</v>
+        <v>399.1300962386066</v>
       </c>
       <c r="I20">
-        <v>565.83396146383166</v>
+        <v>400.92148896127702</v>
       </c>
       <c r="J20">
-        <v>497.28619293931843</v>
+        <v>443.13309694196153</v>
       </c>
       <c r="K20">
-        <v>368.68422318270018</v>
+        <v>348.19454483269311</v>
       </c>
       <c r="L20">
-        <v>401.10201604492812</v>
+        <v>146.67911169289749</v>
       </c>
       <c r="M20">
-        <v>247.6232090369173</v>
+        <v>79.039758363171472</v>
       </c>
       <c r="N20">
-        <v>307.26348235991912</v>
+        <v>341.86467109003041</v>
       </c>
       <c r="O20">
-        <v>19.02130589960159</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
+        <v>32.272430550738513</v>
+      </c>
+      <c r="X20">
+        <v>60.699558981672652</v>
+      </c>
+      <c r="Y20">
+        <v>146.67911169289749</v>
+      </c>
+      <c r="Z20">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="B21">
-        <v>495</v>
+        <v>21</v>
       </c>
       <c r="C21" t="s">
         <v>16</v>
       </c>
       <c r="D21">
-        <v>38.858369836070679</v>
+        <v>77.899336063102595</v>
       </c>
       <c r="E21">
-        <v>23.003241880869538</v>
+        <v>133.0433501484159</v>
       </c>
       <c r="F21">
-        <v>55.529786383888649</v>
+        <v>244.22639878160419</v>
       </c>
       <c r="G21">
-        <v>29.69081823332094</v>
+        <v>26.567574003844118</v>
       </c>
       <c r="H21">
-        <v>373.3529496894771</v>
+        <v>425.51980766516073</v>
       </c>
       <c r="I21">
-        <v>372.97320959068219</v>
+        <v>413.44261080633879</v>
       </c>
       <c r="J21">
-        <v>380.82651312061648</v>
+        <v>449.4966738688878</v>
       </c>
       <c r="K21">
-        <v>399.01944703871101</v>
+        <v>405.34106027925668</v>
       </c>
       <c r="L21">
-        <v>42.167018507148647</v>
+        <v>192.43922175312059</v>
       </c>
       <c r="M21">
-        <v>47.935403518265773</v>
+        <v>240.68931214509649</v>
       </c>
       <c r="N21">
-        <v>28.939664094241479</v>
+        <v>104.9568995869359</v>
       </c>
       <c r="O21">
-        <v>90.152138198962177</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
+        <v>27.027607407580561</v>
+      </c>
+      <c r="X21">
+        <v>77.899336063102595</v>
+      </c>
+      <c r="Y21">
+        <v>192.43922175312059</v>
+      </c>
+      <c r="Z21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="B22">
-        <v>96</v>
+        <v>335</v>
       </c>
       <c r="C22" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D22">
-        <v>32.414671865407158</v>
+        <v>22.197274090792799</v>
       </c>
       <c r="E22">
-        <v>33.564519055947748</v>
+        <v>33.297934879256367</v>
       </c>
       <c r="F22">
-        <v>60.321476631033057</v>
+        <v>42.568472613113883</v>
       </c>
       <c r="G22">
-        <v>18.091963649755549</v>
+        <v>31.327722143945099</v>
       </c>
       <c r="H22">
-        <v>383.9118653614496</v>
+        <v>366.07114517867598</v>
       </c>
       <c r="I22">
-        <v>394.86238272033529</v>
+        <v>372.00312551132578</v>
       </c>
       <c r="J22">
-        <v>364.16552552936167</v>
+        <v>336.37134038928968</v>
       </c>
       <c r="K22">
-        <v>370.26474052585701</v>
+        <v>401.89676721359422</v>
       </c>
       <c r="L22">
-        <v>46.620381592635447</v>
+        <v>55.31221862647083</v>
       </c>
       <c r="M22">
-        <v>75.458971602803246</v>
+        <v>51.458262650400542</v>
       </c>
       <c r="N22">
-        <v>100.20669343017801</v>
+        <v>35.70037129900021</v>
       </c>
       <c r="O22">
-        <v>20.04588568941692</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
+        <v>92.188929384129608</v>
+      </c>
+      <c r="X22">
+        <v>22.197274090792799</v>
+      </c>
+      <c r="Y22">
+        <v>55.31221862647083</v>
+      </c>
+      <c r="Z22">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="B23">
-        <v>43</v>
+        <v>75</v>
       </c>
       <c r="C23" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D23">
-        <v>157.1695900673632</v>
+        <v>30.51539293609839</v>
       </c>
       <c r="E23">
-        <v>452.26091429252358</v>
+        <v>82.40253240156062</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>57.310576672544023</v>
       </c>
       <c r="G23">
-        <v>11.210362501833741</v>
+        <v>23.465951776886801</v>
       </c>
       <c r="H23">
-        <v>615.41199521940575</v>
+        <v>353.14243573105267</v>
       </c>
       <c r="I23">
-        <v>565.14299075157919</v>
+        <v>298.29014664535418</v>
       </c>
       <c r="J23">
-        <v>0</v>
+        <v>359.74644074030402</v>
       </c>
       <c r="K23">
-        <v>427.6650536975892</v>
+        <v>437.44595277098568</v>
       </c>
       <c r="L23">
-        <v>506.00630905275358</v>
+        <v>138.0198512566518</v>
       </c>
       <c r="M23">
-        <v>439.21143002100348</v>
+        <v>58.247651084665328</v>
       </c>
       <c r="N23">
-        <v>0</v>
+        <v>81.731857712478572</v>
       </c>
       <c r="O23">
-        <v>12.60936602372389</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
+        <v>38.633752856784533</v>
+      </c>
+      <c r="Q23" s="10"/>
+      <c r="R23" s="10"/>
+      <c r="S23" s="10"/>
+      <c r="X23">
+        <v>30.51539293609839</v>
+      </c>
+      <c r="Y23">
+        <v>138.0198512566518</v>
+      </c>
+      <c r="Z23">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="B24">
-        <v>147</v>
+        <v>86</v>
       </c>
       <c r="C24" t="s">
         <v>16</v>
       </c>
       <c r="D24">
-        <v>157.75639828891099</v>
+        <v>15.676860792558641</v>
       </c>
       <c r="E24">
-        <v>209.50239690610761</v>
+        <v>24.95662483006106</v>
       </c>
       <c r="F24">
-        <v>129.9183484252321</v>
+        <v>36.583952298580613</v>
       </c>
       <c r="G24">
-        <v>15.466662288797361</v>
+        <v>73.12951840352693</v>
       </c>
       <c r="H24">
-        <v>399.38009470532103</v>
+        <v>404.67525596252852</v>
       </c>
       <c r="I24">
-        <v>394.69514364353279</v>
+        <v>410.05361250495127</v>
       </c>
       <c r="J24">
-        <v>379.86227938982069</v>
+        <v>373.71512291049578</v>
       </c>
       <c r="K24">
-        <v>347.22455284469203</v>
+        <v>365.21688882470858</v>
       </c>
       <c r="L24">
-        <v>216.89246388962491</v>
+        <v>20.768724111329409</v>
       </c>
       <c r="M24">
-        <v>87.143027401900639</v>
+        <v>31.8442768125439</v>
       </c>
       <c r="N24">
-        <v>163.42557540023401</v>
+        <v>52.741272535144361</v>
       </c>
       <c r="O24">
-        <v>27.679016770206019</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
+        <v>82.359000218931229</v>
+      </c>
+      <c r="Q24" s="10"/>
+      <c r="R24" s="10"/>
+      <c r="S24" s="10"/>
+      <c r="X24">
+        <v>15.676860792558641</v>
+      </c>
+      <c r="Y24">
+        <v>20.768724111329409</v>
+      </c>
+      <c r="Z24">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="B25">
-        <v>78</v>
+        <v>25</v>
       </c>
       <c r="C25" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D25">
-        <v>32.862954557960613</v>
+        <v>58.844800566193008</v>
       </c>
       <c r="E25">
-        <v>29.30766691598058</v>
+        <v>90.615389497732849</v>
       </c>
       <c r="F25">
-        <v>58.327163555998808</v>
+        <v>112.7879927934196</v>
       </c>
       <c r="G25">
-        <v>65.340046700283978</v>
+        <v>19.43876498424979</v>
       </c>
       <c r="H25">
-        <v>314.92141321716002</v>
+        <v>419.13865415251769</v>
       </c>
       <c r="I25">
-        <v>302.2424751889194</v>
+        <v>405.01941746680922</v>
       </c>
       <c r="J25">
-        <v>351.07563311842262</v>
+        <v>390.88814554169801</v>
       </c>
       <c r="K25">
-        <v>464.01438700261582</v>
+        <v>371.66055821416597</v>
       </c>
       <c r="L25">
-        <v>38.270074263971317</v>
+        <v>85.202386519051473</v>
       </c>
       <c r="M25">
-        <v>37.265863386800177</v>
+        <v>110.4695478458745</v>
       </c>
       <c r="N25">
-        <v>192.09464362385529</v>
+        <v>83.055424716918992</v>
       </c>
       <c r="O25">
-        <v>132.8810109534945</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
+        <v>20.743103523213659</v>
+      </c>
+      <c r="Q25" s="10"/>
+      <c r="R25" s="10"/>
+      <c r="S25" s="10"/>
+      <c r="X25">
+        <v>58.844800566193008</v>
+      </c>
+      <c r="Y25">
+        <v>85.202386519051473</v>
+      </c>
+      <c r="Z25">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="B26">
-        <v>38</v>
+        <v>60</v>
       </c>
       <c r="C26" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D26">
-        <v>42.174163843223148</v>
+        <v>48.132329238563791</v>
       </c>
       <c r="E26">
-        <v>53.632066786364483</v>
+        <v>70.18269765958317</v>
       </c>
       <c r="F26">
-        <v>71.73497288331221</v>
+        <v>93.555964526333838</v>
       </c>
       <c r="G26">
-        <v>11.13986017896976</v>
+        <v>10.270982158460781</v>
       </c>
       <c r="H26">
-        <v>424.95132148329611</v>
+        <v>339.50226684665591</v>
       </c>
       <c r="I26">
-        <v>439.62899346820922</v>
+        <v>341.78751798734248</v>
       </c>
       <c r="J26">
-        <v>435.98867231614668</v>
+        <v>358.56064050986407</v>
       </c>
       <c r="K26">
-        <v>431.02577304273382</v>
+        <v>361.57224353690611</v>
       </c>
       <c r="L26">
-        <v>48.193870627407797</v>
+        <v>112.87910589847991</v>
       </c>
       <c r="M26">
-        <v>83.177419896509122</v>
+        <v>110.6236295208824</v>
       </c>
       <c r="N26">
-        <v>105.83908579791429</v>
+        <v>170.8385032445826</v>
       </c>
       <c r="O26">
-        <v>12.17441727699982</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+        <v>11.35357425855055</v>
+      </c>
+      <c r="Q26" s="10"/>
+      <c r="R26" s="10"/>
+      <c r="S26" s="10"/>
+      <c r="X26">
+        <v>48.132329238563791</v>
+      </c>
+      <c r="Y26">
+        <v>112.87910589847991</v>
+      </c>
+      <c r="Z26">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="B27">
-        <v>14</v>
+        <v>134</v>
       </c>
       <c r="C27" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D27">
-        <v>126.9799700740049</v>
+        <v>24.067675084096521</v>
       </c>
       <c r="E27">
-        <v>162.07028163118969</v>
+        <v>45.551283034671343</v>
       </c>
       <c r="F27">
-        <v>164.57093868050831</v>
+        <v>35.332196394666482</v>
       </c>
       <c r="G27">
-        <v>15.991463717523359</v>
+        <v>35.330973983850477</v>
       </c>
       <c r="H27">
-        <v>523.20873505511861</v>
+        <v>353.23026285364409</v>
       </c>
       <c r="I27">
-        <v>543.28250605443202</v>
+        <v>436.12092907185018</v>
       </c>
       <c r="J27">
-        <v>412.38703977632491</v>
+        <v>283.82788317154279</v>
       </c>
       <c r="K27">
-        <v>350.38293551849108</v>
+        <v>299.94876454097539</v>
       </c>
       <c r="L27">
-        <v>276.08480721054008</v>
+        <v>100.1706393901803</v>
       </c>
       <c r="M27">
-        <v>382.38921548386458</v>
+        <v>133.85366595632371</v>
       </c>
       <c r="N27">
-        <v>287.95877341887308</v>
+        <v>55.075690143004557</v>
       </c>
       <c r="O27">
-        <v>19.251661139323598</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
+        <v>108.35361813077991</v>
+      </c>
+      <c r="Q27" s="10"/>
+      <c r="R27" s="10"/>
+      <c r="S27" s="10"/>
+      <c r="X27">
+        <v>24.067675084096521</v>
+      </c>
+      <c r="Y27">
+        <v>100.1706393901803</v>
+      </c>
+      <c r="Z27">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="B28">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="C28" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D28">
-        <v>55.291681493457482</v>
+        <v>26.945203084574931</v>
       </c>
       <c r="E28">
-        <v>66.679942252024688</v>
+        <v>22.423372885417809</v>
       </c>
       <c r="F28">
-        <v>45.261438386854543</v>
+        <v>54.469166827601782</v>
       </c>
       <c r="G28">
-        <v>15.383426445738831</v>
+        <v>38.667004176022338</v>
       </c>
       <c r="H28">
-        <v>384.91023860758651</v>
+        <v>399.44864226640658</v>
       </c>
       <c r="I28">
-        <v>310.63575289638578</v>
+        <v>402.10594182481708</v>
       </c>
       <c r="J28">
-        <v>376.86666337313551</v>
+        <v>422.90907304513883</v>
       </c>
       <c r="K28">
-        <v>511.85507380384217</v>
+        <v>435.5821677117242</v>
       </c>
       <c r="L28">
-        <v>91.004292001720501</v>
+        <v>33.030887251015379</v>
       </c>
       <c r="M28">
-        <v>80.34943319202263</v>
+        <v>24.87777722703504</v>
       </c>
       <c r="N28">
-        <v>97.041583145992277</v>
+        <v>137.1861931594716</v>
       </c>
       <c r="O28">
-        <v>22.001519553737559</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
+        <v>51.931955676615154</v>
+      </c>
+      <c r="Q28" s="10"/>
+      <c r="R28" s="10"/>
+      <c r="S28" s="10"/>
+      <c r="X28">
+        <v>26.945203084574931</v>
+      </c>
+      <c r="Y28">
+        <v>33.030887251015379</v>
+      </c>
+      <c r="Z28">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="B29">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="C29" t="s">
         <v>16</v>
       </c>
       <c r="D29">
-        <v>26.514968970004919</v>
+        <v>109.73707886519161</v>
       </c>
       <c r="E29">
-        <v>27.930890454349871</v>
+        <v>261.13776919725211</v>
       </c>
       <c r="F29">
-        <v>42.841332240449987</v>
+        <v>226.34339234893409</v>
       </c>
       <c r="G29">
-        <v>27.092258521692589</v>
+        <v>11.605070703761021</v>
       </c>
       <c r="H29">
-        <v>401.24140347035029</v>
+        <v>489.83552856883159</v>
       </c>
       <c r="I29">
-        <v>390.58785075394218</v>
+        <v>261.13776919725211</v>
       </c>
       <c r="J29">
-        <v>385.15892322945092</v>
+        <v>496.22675882897698</v>
       </c>
       <c r="K29">
-        <v>376.91842529035341</v>
+        <v>505.79575177022258</v>
       </c>
       <c r="L29">
-        <v>29.380245318894701</v>
+        <v>189.9556814939302</v>
       </c>
       <c r="M29">
-        <v>29.05871847571445</v>
+        <v>57.734343332197007</v>
       </c>
       <c r="N29">
-        <v>44.779463616152093</v>
+        <v>356.04000020375452</v>
       </c>
       <c r="O29">
-        <v>28.10572963842079</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
+        <v>17.127483308572391</v>
+      </c>
+      <c r="Q29" s="10"/>
+      <c r="R29" s="10"/>
+      <c r="S29" s="10"/>
+      <c r="X29">
+        <v>109.73707886519161</v>
+      </c>
+      <c r="Y29">
+        <v>189.9556814939302</v>
+      </c>
+      <c r="Z29">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="B30">
-        <v>100</v>
+        <v>18</v>
       </c>
       <c r="C30" t="s">
         <v>16</v>
       </c>
       <c r="D30">
-        <v>24.227225068400369</v>
+        <v>92.342254873128724</v>
       </c>
       <c r="E30">
-        <v>35.480122730762197</v>
+        <v>112.6809640903937</v>
       </c>
       <c r="F30">
-        <v>37.736667367152322</v>
+        <v>52.144533677607292</v>
       </c>
       <c r="G30">
-        <v>21.86016814579628</v>
+        <v>17.5963816071284</v>
       </c>
       <c r="H30">
-        <v>353.42302267168043</v>
+        <v>320.04098190997871</v>
       </c>
       <c r="I30">
-        <v>357.69953615911032</v>
+        <v>338.44022593256699</v>
       </c>
       <c r="J30">
-        <v>341.00883908011042</v>
+        <v>355.71090011217842</v>
       </c>
       <c r="K30">
-        <v>360.39677598267832</v>
+        <v>371.69817777284209</v>
       </c>
       <c r="L30">
-        <v>29.87344806809881</v>
+        <v>99.709613853874075</v>
       </c>
       <c r="M30">
-        <v>44.057606804907749</v>
+        <v>120.190214958013</v>
       </c>
       <c r="N30">
-        <v>55.444262774132113</v>
+        <v>55.175647895780898</v>
       </c>
       <c r="O30">
-        <v>23.691980427160729</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
+        <v>19.168394322717209</v>
+      </c>
+      <c r="Q30" s="10"/>
+      <c r="R30" s="10"/>
+      <c r="S30" s="10"/>
+      <c r="X30">
+        <v>92.342254873128724</v>
+      </c>
+      <c r="Y30">
+        <v>99.709613853874075</v>
+      </c>
+      <c r="Z30">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="B31">
-        <v>48</v>
+        <v>127</v>
       </c>
       <c r="C31" t="s">
         <v>16</v>
       </c>
       <c r="D31">
-        <v>26.98944663668691</v>
+        <v>145.79226907872891</v>
       </c>
       <c r="E31">
-        <v>33.895915994301347</v>
+        <v>119.243151091578</v>
       </c>
       <c r="F31">
-        <v>37.256565678364083</v>
+        <v>227.21588577516371</v>
       </c>
       <c r="G31">
-        <v>11.128145913861321</v>
+        <v>18.594188650084359</v>
       </c>
       <c r="H31">
-        <v>312.23451990534687</v>
+        <v>416.81494970243853</v>
       </c>
       <c r="I31">
-        <v>355.43723262233408</v>
+        <v>398.62160931867243</v>
       </c>
       <c r="J31">
-        <v>308.78392064557579</v>
+        <v>405.1202850903386</v>
       </c>
       <c r="K31">
-        <v>333.21999986488811</v>
+        <v>423.23411992886292</v>
       </c>
       <c r="L31">
-        <v>37.71408536963763</v>
+        <v>44.02448729446192</v>
       </c>
       <c r="M31">
-        <v>92.632080716457835</v>
+        <v>49.661683396420337</v>
       </c>
       <c r="N31">
-        <v>79.273890310224957</v>
+        <v>36.532336388861793</v>
       </c>
       <c r="O31">
-        <v>11.31663605866877</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
+        <v>21.252794080640541</v>
+      </c>
+      <c r="X31">
+        <v>145.79226907872891</v>
+      </c>
+      <c r="Y31">
+        <v>44.02448729446192</v>
+      </c>
+      <c r="Z31">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>47</v>
+        <v>71</v>
       </c>
       <c r="B32">
-        <v>71</v>
+        <v>124</v>
       </c>
       <c r="C32" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D32">
-        <v>25.458334546352621</v>
+        <v>45.350272058957557</v>
       </c>
       <c r="E32">
-        <v>27.56141082978565</v>
+        <v>58.700289697901027</v>
       </c>
       <c r="F32">
-        <v>44.432831365430992</v>
+        <v>77.516673409048039</v>
       </c>
       <c r="G32">
-        <v>26.762162283832058</v>
+        <v>20.95128439121024</v>
       </c>
       <c r="H32">
-        <v>343.01850166562031</v>
+        <v>406.9102608456771</v>
       </c>
       <c r="I32">
-        <v>348.93211868555733</v>
+        <v>406.78224130167632</v>
       </c>
       <c r="J32">
-        <v>344.02351834087563</v>
+        <v>405.86090497093301</v>
       </c>
       <c r="K32">
-        <v>378.48732880361229</v>
+        <v>392.22590157363243</v>
       </c>
       <c r="L32">
-        <v>34.472081962895253</v>
+        <v>93.83477160384281</v>
       </c>
       <c r="M32">
-        <v>34.536297047842353</v>
+        <v>52.808598539760723</v>
       </c>
       <c r="N32">
-        <v>96.52038314724787</v>
+        <v>59.330492886414532</v>
       </c>
       <c r="O32">
-        <v>32.105890646351718</v>
-      </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
+        <v>24.393175379022772</v>
+      </c>
+      <c r="X32">
+        <v>45.350272058957557</v>
+      </c>
+      <c r="Y32">
+        <v>93.83477160384281</v>
+      </c>
+      <c r="Z32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>48</v>
+        <v>72</v>
       </c>
       <c r="B33">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="C33" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D33">
-        <v>36.115000207075248</v>
+        <v>53.222482281183758</v>
       </c>
       <c r="E33">
-        <v>61.930988311744741</v>
+        <v>63.298469519821687</v>
       </c>
       <c r="F33">
-        <v>52.7106501263127</v>
+        <v>65.863865836910421</v>
       </c>
       <c r="G33">
-        <v>20.18191692693793</v>
+        <v>12.90970715156589</v>
       </c>
       <c r="H33">
-        <v>362.78025391217813</v>
+        <v>376.16375212277097</v>
       </c>
       <c r="I33">
-        <v>317.62034077392468</v>
+        <v>368.43490525946271</v>
       </c>
       <c r="J33">
-        <v>366.11102814828041</v>
+        <v>378.11113342938671</v>
       </c>
       <c r="K33">
-        <v>381.06058054605012</v>
+        <v>381.35022296080172</v>
       </c>
       <c r="L33">
-        <v>39.47815909350502</v>
+        <v>69.126273897807906</v>
       </c>
       <c r="M33">
-        <v>104.0359985074374</v>
+        <v>114.8944866491285</v>
       </c>
       <c r="N33">
-        <v>54.626847894740351</v>
+        <v>137.98814458622681</v>
       </c>
       <c r="O33">
-        <v>20.28409136690885</v>
-      </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
+        <v>13.40732613888288</v>
+      </c>
+      <c r="X33">
+        <v>53.222482281183758</v>
+      </c>
+      <c r="Y33">
+        <v>69.126273897807906</v>
+      </c>
+      <c r="Z33">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>49</v>
+        <v>73</v>
       </c>
       <c r="B34">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="C34" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D34">
-        <v>27.141428170684911</v>
+        <v>35.845989483527148</v>
       </c>
       <c r="E34">
-        <v>74.205514562532983</v>
+        <v>55.900912828113093</v>
       </c>
       <c r="F34">
-        <v>50.795139394736069</v>
+        <v>41.448538191005717</v>
       </c>
       <c r="G34">
-        <v>13.876890987594409</v>
+        <v>27.37782151530843</v>
       </c>
       <c r="H34">
-        <v>437.29671802253648</v>
+        <v>334.77724853747748</v>
       </c>
       <c r="I34">
-        <v>450.16820371038369</v>
+        <v>305.6194814065322</v>
       </c>
       <c r="J34">
-        <v>424.48849183203077</v>
+        <v>356.88648271383181</v>
       </c>
       <c r="K34">
-        <v>362.98327767688102</v>
+        <v>410.83967206156052</v>
       </c>
       <c r="L34">
-        <v>54.607081730162797</v>
+        <v>40.105904559271707</v>
       </c>
       <c r="M34">
-        <v>104.1460995556302</v>
+        <v>104.1427539838388</v>
       </c>
       <c r="N34">
-        <v>88.632730599537496</v>
+        <v>80.332767710706236</v>
       </c>
       <c r="O34">
-        <v>14.59337143572642</v>
-      </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.35">
+        <v>32.365358351714853</v>
+      </c>
+      <c r="X34">
+        <v>35.845989483527148</v>
+      </c>
+      <c r="Y34">
+        <v>40.105904559271707</v>
+      </c>
+      <c r="Z34">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="B35">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C35" t="s">
         <v>22</v>
       </c>
       <c r="D35">
-        <v>38.76855960345658</v>
-      </c>
-      <c r="E35">
-        <v>58.160357767798907</v>
+        <v>95.952061780353603</v>
       </c>
       <c r="F35">
-        <v>63.131696409314458</v>
+        <v>191.8574369369565</v>
       </c>
       <c r="G35">
-        <v>27.992737517673032</v>
+        <v>10.28284606445969</v>
       </c>
       <c r="H35">
-        <v>309.89218013465592</v>
-      </c>
-      <c r="I35">
-        <v>336.03554179181032</v>
+        <v>482.95669182112181</v>
       </c>
       <c r="J35">
-        <v>330.44036703039092</v>
+        <v>362.76347828603468</v>
       </c>
       <c r="K35">
-        <v>386.89860148852949</v>
+        <v>446.3343062424355</v>
       </c>
       <c r="L35">
-        <v>45.601378712452117</v>
-      </c>
-      <c r="M35">
-        <v>71.29228681988954</v>
+        <v>289.24872066023192</v>
       </c>
       <c r="N35">
-        <v>149.63878938188569</v>
+        <v>214.6767046368949</v>
       </c>
       <c r="O35">
-        <v>28.019281070537531</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.35">
+        <v>10.28284606445969</v>
+      </c>
+      <c r="X35">
+        <v>95.952061780353603</v>
+      </c>
+      <c r="Y35">
+        <v>289.24872066023192</v>
+      </c>
+      <c r="Z35">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="B36">
-        <v>77</v>
+        <v>29</v>
       </c>
       <c r="C36" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D36">
-        <v>60.699558981672652</v>
+        <v>91.71700113373214</v>
       </c>
       <c r="E36">
-        <v>31.472697816142691</v>
+        <v>50.58835564570748</v>
       </c>
       <c r="F36">
-        <v>208.58516339246131</v>
+        <v>573.29576775519558</v>
       </c>
       <c r="G36">
-        <v>26.271065972465401</v>
+        <v>79.245818219534939</v>
       </c>
       <c r="H36">
-        <v>399.1300962386066</v>
+        <v>403.76236488191728</v>
       </c>
       <c r="I36">
-        <v>400.92148896127702</v>
+        <v>465.33915893749509</v>
       </c>
       <c r="J36">
-        <v>443.13309694196153</v>
+        <v>573.29576775519558</v>
       </c>
       <c r="K36">
-        <v>348.19454483269311</v>
+        <v>370.05124866902253</v>
       </c>
       <c r="L36">
-        <v>146.67911169289749</v>
+        <v>177.05480894775809</v>
       </c>
       <c r="M36">
-        <v>79.039758363171472</v>
+        <v>103.8138812333322</v>
       </c>
       <c r="N36">
-        <v>341.86467109003041</v>
+        <v>15.864217850243991</v>
       </c>
       <c r="O36">
-        <v>32.272430550738513</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.35">
+        <v>104.282643969308</v>
+      </c>
+      <c r="X36">
+        <v>91.71700113373214</v>
+      </c>
+      <c r="Y36">
+        <v>177.05480894775809</v>
+      </c>
+      <c r="Z36">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="B37">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="C37" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D37">
-        <v>77.899336063102595</v>
+        <v>127.0414892215851</v>
       </c>
       <c r="E37">
-        <v>133.0433501484159</v>
+        <v>161.79046065770581</v>
       </c>
       <c r="F37">
-        <v>244.22639878160419</v>
+        <v>193.4390885246533</v>
       </c>
       <c r="G37">
-        <v>26.567574003844118</v>
+        <v>16.599355594149358</v>
       </c>
       <c r="H37">
-        <v>425.51980766516073</v>
+        <v>444.57000559024959</v>
       </c>
       <c r="I37">
-        <v>413.44261080633879</v>
+        <v>469.29795805113702</v>
       </c>
       <c r="J37">
-        <v>449.4966738688878</v>
+        <v>477.60802690206509</v>
       </c>
       <c r="K37">
-        <v>405.34106027925668</v>
+        <v>396.91837570010819</v>
       </c>
       <c r="L37">
-        <v>192.43922175312059</v>
+        <v>234.37095667492471</v>
       </c>
       <c r="M37">
-        <v>240.68931214509649</v>
+        <v>263.16988534515559</v>
       </c>
       <c r="N37">
-        <v>104.9568995869359</v>
+        <v>264.95906826024179</v>
       </c>
       <c r="O37">
-        <v>27.027607407580561</v>
-      </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.35">
+        <v>19.25326026909352</v>
+      </c>
+      <c r="X37">
+        <v>127.0414892215851</v>
+      </c>
+      <c r="Y37">
+        <v>234.37095667492471</v>
+      </c>
+      <c r="Z37">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="B38">
-        <v>335</v>
+        <v>42</v>
       </c>
       <c r="C38" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D38">
-        <v>22.197274090792799</v>
+        <v>56.611725681597093</v>
       </c>
       <c r="E38">
-        <v>33.297934879256367</v>
+        <v>139.1030672878758</v>
       </c>
       <c r="F38">
-        <v>42.568472613113883</v>
+        <v>91.895401500037494</v>
       </c>
       <c r="G38">
-        <v>31.327722143945099</v>
+        <v>24.01054211217313</v>
       </c>
       <c r="H38">
-        <v>366.07114517867598</v>
+        <v>406.31802223501558</v>
       </c>
       <c r="I38">
-        <v>372.00312551132578</v>
+        <v>461.4504742414772</v>
       </c>
       <c r="J38">
-        <v>336.37134038928968</v>
+        <v>423.70214873900591</v>
       </c>
       <c r="K38">
-        <v>401.89676721359422</v>
+        <v>396.58512384641921</v>
       </c>
       <c r="L38">
-        <v>55.31221862647083</v>
+        <v>82.57993141699049</v>
       </c>
       <c r="M38">
-        <v>51.458262650400542</v>
+        <v>289.25155042577393</v>
       </c>
       <c r="N38">
-        <v>35.70037129900021</v>
+        <v>240.02224576808149</v>
       </c>
       <c r="O38">
-        <v>92.188929384129608</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.35">
+        <v>32.060364125303259</v>
+      </c>
+      <c r="X38">
+        <v>56.611725681597093</v>
+      </c>
+      <c r="Y38">
+        <v>82.57993141699049</v>
+      </c>
+      <c r="Z38">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="B39">
-        <v>75</v>
+        <v>458</v>
       </c>
       <c r="C39" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D39">
-        <v>30.51539293609839</v>
+        <v>65.001757273467902</v>
       </c>
       <c r="E39">
-        <v>82.40253240156062</v>
+        <v>43.860218685961733</v>
       </c>
       <c r="F39">
-        <v>57.310576672544023</v>
+        <v>92.983017447037724</v>
       </c>
       <c r="G39">
-        <v>23.465951776886801</v>
+        <v>17.231497919734071</v>
       </c>
       <c r="H39">
-        <v>353.14243573105267</v>
+        <v>345.52684228687423</v>
       </c>
       <c r="I39">
-        <v>298.29014664535418</v>
+        <v>340.95971503899079</v>
       </c>
       <c r="J39">
-        <v>359.74644074030402</v>
+        <v>349.27117327367802</v>
       </c>
       <c r="K39">
-        <v>437.44595277098568</v>
+        <v>408.81734039456319</v>
       </c>
       <c r="L39">
-        <v>138.0198512566518</v>
+        <v>36.55900717081883</v>
       </c>
       <c r="M39">
-        <v>58.247651084665328</v>
+        <v>32.989309807573413</v>
       </c>
       <c r="N39">
-        <v>81.731857712478572</v>
+        <v>25.83869576242795</v>
       </c>
       <c r="O39">
-        <v>38.633752856784533</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.35">
+        <v>27.028190687332021</v>
+      </c>
+      <c r="X39">
+        <v>65.001757273467902</v>
+      </c>
+      <c r="Y39">
+        <v>36.55900717081883</v>
+      </c>
+      <c r="Z39">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="B40">
-        <v>86</v>
+        <v>416</v>
       </c>
       <c r="C40" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D40">
-        <v>15.676860792558641</v>
+        <v>83.028796498862903</v>
       </c>
       <c r="E40">
-        <v>24.95662483006106</v>
+        <v>71.287098259342031</v>
       </c>
       <c r="F40">
-        <v>36.583952298580613</v>
+        <v>130.9636023752484</v>
       </c>
       <c r="G40">
-        <v>73.12951840352693</v>
+        <v>15.836556562469269</v>
       </c>
       <c r="H40">
-        <v>404.67525596252852</v>
+        <v>398.04948882641889</v>
       </c>
       <c r="I40">
-        <v>410.05361250495127</v>
+        <v>393.38916107738578</v>
       </c>
       <c r="J40">
-        <v>373.71512291049578</v>
+        <v>401.22822159322033</v>
       </c>
       <c r="K40">
-        <v>365.21688882470858</v>
+        <v>368.02768399560898</v>
       </c>
       <c r="L40">
-        <v>20.768724111329409</v>
+        <v>59.702356290752988</v>
       </c>
       <c r="M40">
-        <v>31.8442768125439</v>
+        <v>51.002124872064037</v>
       </c>
       <c r="N40">
-        <v>52.741272535144361</v>
+        <v>64.609602756275436</v>
       </c>
       <c r="O40">
-        <v>82.359000218931229</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.35">
+        <v>20.955192969868751</v>
+      </c>
+      <c r="X40">
+        <v>83.028796498862903</v>
+      </c>
+      <c r="Y40">
+        <v>59.702356290752988</v>
+      </c>
+      <c r="Z40">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>56</v>
+        <v>37</v>
       </c>
       <c r="B41">
-        <v>25</v>
+        <v>96</v>
       </c>
       <c r="C41" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D41">
-        <v>58.844800566193008</v>
+        <v>32.414671865407158</v>
       </c>
       <c r="E41">
-        <v>90.615389497732849</v>
+        <v>33.564519055947748</v>
       </c>
       <c r="F41">
-        <v>112.7879927934196</v>
+        <v>60.321476631033057</v>
       </c>
       <c r="G41">
-        <v>19.43876498424979</v>
+        <v>18.091963649755549</v>
       </c>
       <c r="H41">
-        <v>419.13865415251769</v>
+        <v>383.9118653614496</v>
       </c>
       <c r="I41">
-        <v>405.01941746680922</v>
+        <v>394.86238272033529</v>
       </c>
       <c r="J41">
-        <v>390.88814554169801</v>
+        <v>364.16552552936167</v>
       </c>
       <c r="K41">
-        <v>371.66055821416597</v>
+        <v>370.26474052585701</v>
       </c>
       <c r="L41">
-        <v>85.202386519051473</v>
+        <v>46.620381592635447</v>
       </c>
       <c r="M41">
-        <v>110.4695478458745</v>
+        <v>75.458971602803246</v>
       </c>
       <c r="N41">
-        <v>83.055424716918992</v>
+        <v>100.20669343017801</v>
       </c>
       <c r="O41">
-        <v>20.743103523213659</v>
-      </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.35">
+        <v>20.04588568941692</v>
+      </c>
+      <c r="X41">
+        <v>32.414671865407158</v>
+      </c>
+      <c r="Y41">
+        <v>46.620381592635447</v>
+      </c>
+      <c r="Z41">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="B42">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C42" t="s">
         <v>22</v>
       </c>
       <c r="D42">
-        <v>102.2273523737079</v>
+        <v>157.1695900673632</v>
       </c>
       <c r="E42">
-        <v>94.377073315763724</v>
-      </c>
-      <c r="F42">
-        <v>248.7240832590131</v>
+        <v>452.26091429252358</v>
       </c>
       <c r="G42">
-        <v>14.764428597060119</v>
+        <v>11.210362501833741</v>
       </c>
       <c r="H42">
-        <v>509.11392537154251</v>
+        <v>615.41199521940575</v>
       </c>
       <c r="I42">
-        <v>444.5394387903192</v>
-      </c>
-      <c r="J42">
-        <v>452.98134172715493</v>
+        <v>565.14299075157919</v>
       </c>
       <c r="K42">
-        <v>437.48115353530579</v>
+        <v>427.6650536975892</v>
       </c>
       <c r="L42">
-        <v>376.3303565989475</v>
+        <v>506.00630905275358</v>
       </c>
       <c r="M42">
-        <v>222.8020800528106</v>
-      </c>
-      <c r="N42">
-        <v>166.23762217502701</v>
+        <v>439.21143002100348</v>
       </c>
       <c r="O42">
-        <v>15.344741114274161</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.35">
+        <v>12.60936602372389</v>
+      </c>
+      <c r="X42">
+        <v>157.1695900673632</v>
+      </c>
+      <c r="Y42">
+        <v>506.00630905275358</v>
+      </c>
+      <c r="Z42">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="B43">
-        <v>111</v>
+        <v>78</v>
       </c>
       <c r="C43" t="s">
         <v>22</v>
       </c>
       <c r="D43">
-        <v>39.531777047755639</v>
+        <v>32.862954557960613</v>
       </c>
       <c r="E43">
-        <v>68.82993429858297</v>
+        <v>29.30766691598058</v>
       </c>
       <c r="F43">
-        <v>78.35808245663813</v>
+        <v>58.327163555998808</v>
       </c>
       <c r="G43">
-        <v>88.061706532621713</v>
+        <v>65.340046700283978</v>
       </c>
       <c r="H43">
-        <v>328.38018664395059</v>
+        <v>314.92141321716002</v>
       </c>
       <c r="I43">
-        <v>304.35343389705952</v>
+        <v>302.2424751889194</v>
       </c>
       <c r="J43">
-        <v>323.05239826335497</v>
+        <v>351.07563311842262</v>
       </c>
       <c r="K43">
-        <v>425.28636284344708</v>
+        <v>464.01438700261582</v>
       </c>
       <c r="L43">
-        <v>103.178598349591</v>
+        <v>38.270074263971317</v>
       </c>
       <c r="M43">
-        <v>30.04465215964467</v>
+        <v>37.265863386800177</v>
       </c>
       <c r="N43">
-        <v>52.563559191054011</v>
+        <v>192.09464362385529</v>
       </c>
       <c r="O43">
-        <v>114.3666958345908</v>
-      </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.35">
+        <v>132.8810109534945</v>
+      </c>
+      <c r="X43">
+        <v>32.862954557960613</v>
+      </c>
+      <c r="Y43">
+        <v>38.270074263971317</v>
+      </c>
+      <c r="Z43">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="B44">
-        <v>174</v>
+        <v>38</v>
       </c>
       <c r="C44" t="s">
         <v>22</v>
       </c>
       <c r="D44">
-        <v>365.3432181055515</v>
+        <v>42.174163843223148</v>
       </c>
       <c r="E44">
-        <v>0</v>
+        <v>53.632066786364483</v>
       </c>
       <c r="F44">
-        <v>589.78607001776163</v>
+        <v>71.73497288331221</v>
       </c>
       <c r="G44">
-        <v>9.0162709181267644</v>
+        <v>11.13986017896976</v>
       </c>
       <c r="H44">
-        <v>620.04476798631129</v>
+        <v>424.95132148329611</v>
       </c>
       <c r="I44">
-        <v>0</v>
+        <v>439.62899346820922</v>
       </c>
       <c r="J44">
-        <v>623.47095650546771</v>
+        <v>435.98867231614668</v>
       </c>
       <c r="K44">
-        <v>398.00357604739531</v>
+        <v>431.02577304273382</v>
       </c>
       <c r="L44">
-        <v>219.67073614440551</v>
+        <v>48.193870627407797</v>
       </c>
       <c r="M44">
-        <v>0</v>
+        <v>83.177419896509122</v>
       </c>
       <c r="N44">
-        <v>108.977655843035</v>
+        <v>105.83908579791429</v>
       </c>
       <c r="O44">
-        <v>11.44303999411494</v>
-      </c>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.35">
+        <v>12.17441727699982</v>
+      </c>
+      <c r="X44">
+        <v>42.174163843223148</v>
+      </c>
+      <c r="Y44">
+        <v>48.193870627407797</v>
+      </c>
+      <c r="Z44">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="B45">
-        <v>73</v>
+        <v>14</v>
       </c>
       <c r="C45" t="s">
         <v>22</v>
       </c>
       <c r="D45">
-        <v>49.727587386255557</v>
+        <v>126.9799700740049</v>
       </c>
       <c r="E45">
-        <v>95.758881643316855</v>
+        <v>162.07028163118969</v>
       </c>
       <c r="F45">
-        <v>91.643737142682156</v>
+        <v>164.57093868050831</v>
       </c>
       <c r="G45">
-        <v>32.109877716184577</v>
+        <v>15.991463717523359</v>
       </c>
       <c r="H45">
-        <v>404.99950839556197</v>
+        <v>523.20873505511861</v>
       </c>
       <c r="I45">
-        <v>407.03622005894118</v>
+        <v>543.28250605443202</v>
       </c>
       <c r="J45">
-        <v>384.84750083257723</v>
+        <v>412.38703977632491</v>
       </c>
       <c r="K45">
-        <v>473.64106558435049</v>
+        <v>350.38293551849108</v>
       </c>
       <c r="L45">
-        <v>105.7829253801773</v>
+        <v>276.08480721054008</v>
       </c>
       <c r="M45">
-        <v>214.14197337529961</v>
+        <v>382.38921548386458</v>
       </c>
       <c r="N45">
-        <v>175.71428013326999</v>
+        <v>287.95877341887308</v>
       </c>
       <c r="O45">
-        <v>37.910314583794097</v>
-      </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.35">
+        <v>19.251661139323598</v>
+      </c>
+      <c r="X45">
+        <v>126.9799700740049</v>
+      </c>
+      <c r="Y45">
+        <v>276.08480721054008</v>
+      </c>
+      <c r="Z45">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="B46">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="C46" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D46">
-        <v>48.132329238563791</v>
+        <v>55.291681493457482</v>
       </c>
       <c r="E46">
-        <v>70.18269765958317</v>
+        <v>66.679942252024688</v>
       </c>
       <c r="F46">
-        <v>93.555964526333838</v>
+        <v>45.261438386854543</v>
       </c>
       <c r="G46">
-        <v>10.270982158460781</v>
+        <v>15.383426445738831</v>
       </c>
       <c r="H46">
-        <v>339.50226684665591</v>
+        <v>384.91023860758651</v>
       </c>
       <c r="I46">
-        <v>341.78751798734248</v>
+        <v>310.63575289638578</v>
       </c>
       <c r="J46">
-        <v>358.56064050986407</v>
+        <v>376.86666337313551</v>
       </c>
       <c r="K46">
-        <v>361.57224353690611</v>
+        <v>511.85507380384217</v>
       </c>
       <c r="L46">
-        <v>112.87910589847991</v>
+        <v>91.004292001720501</v>
       </c>
       <c r="M46">
-        <v>110.6236295208824</v>
+        <v>80.34943319202263</v>
       </c>
       <c r="N46">
-        <v>170.8385032445826</v>
+        <v>97.041583145992277</v>
       </c>
       <c r="O46">
-        <v>11.35357425855055</v>
-      </c>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.35">
+        <v>22.001519553737559</v>
+      </c>
+      <c r="X46">
+        <v>55.291681493457482</v>
+      </c>
+      <c r="Y46">
+        <v>91.004292001720501</v>
+      </c>
+      <c r="Z46">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="B47">
-        <v>27</v>
+        <v>71</v>
       </c>
       <c r="C47" t="s">
         <v>22</v>
       </c>
       <c r="D47">
-        <v>23.646259520680751</v>
+        <v>25.458334546352621</v>
       </c>
       <c r="E47">
-        <v>23.301729159894919</v>
+        <v>27.56141082978565</v>
       </c>
       <c r="F47">
-        <v>32.020454442657062</v>
+        <v>44.432831365430992</v>
       </c>
       <c r="G47">
-        <v>29.24683532529318</v>
+        <v>26.762162283832058</v>
       </c>
       <c r="H47">
-        <v>412.25009682312958</v>
+        <v>343.01850166562031</v>
       </c>
       <c r="I47">
-        <v>403.94176964511178</v>
+        <v>348.93211868555733</v>
       </c>
       <c r="J47">
-        <v>384.67230012765248</v>
+        <v>344.02351834087563</v>
       </c>
       <c r="K47">
-        <v>381.49650965448711</v>
+        <v>378.48732880361229</v>
       </c>
       <c r="L47">
-        <v>24.738052884723761</v>
+        <v>34.472081962895253</v>
       </c>
       <c r="M47">
-        <v>23.89989208087173</v>
+        <v>34.536297047842353</v>
       </c>
       <c r="N47">
-        <v>38.701299967223129</v>
+        <v>96.52038314724787</v>
       </c>
       <c r="O47">
-        <v>29.761725902459961</v>
-      </c>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.35">
+        <v>32.105890646351718</v>
+      </c>
+      <c r="X47">
+        <v>25.458334546352621</v>
+      </c>
+      <c r="Y47">
+        <v>34.472081962895253</v>
+      </c>
+      <c r="Z47">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="B48">
-        <v>134</v>
+        <v>20</v>
       </c>
       <c r="C48" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D48">
-        <v>24.067675084096521</v>
+        <v>36.115000207075248</v>
       </c>
       <c r="E48">
-        <v>45.551283034671343</v>
+        <v>61.930988311744741</v>
       </c>
       <c r="F48">
-        <v>35.332196394666482</v>
+        <v>52.7106501263127</v>
       </c>
       <c r="G48">
-        <v>35.330973983850477</v>
+        <v>20.18191692693793</v>
       </c>
       <c r="H48">
-        <v>353.23026285364409</v>
+        <v>362.78025391217813</v>
       </c>
       <c r="I48">
-        <v>436.12092907185018</v>
+        <v>317.62034077392468</v>
       </c>
       <c r="J48">
-        <v>283.82788317154279</v>
+        <v>366.11102814828041</v>
       </c>
       <c r="K48">
-        <v>299.94876454097539</v>
+        <v>381.06058054605012</v>
       </c>
       <c r="L48">
-        <v>100.1706393901803</v>
+        <v>39.47815909350502</v>
       </c>
       <c r="M48">
-        <v>133.85366595632371</v>
+        <v>104.0359985074374</v>
       </c>
       <c r="N48">
-        <v>55.075690143004557</v>
+        <v>54.626847894740351</v>
       </c>
       <c r="O48">
-        <v>108.35361813077991</v>
-      </c>
-    </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.35">
+        <v>20.28409136690885</v>
+      </c>
+      <c r="X48">
+        <v>36.115000207075248</v>
+      </c>
+      <c r="Y48">
+        <v>39.47815909350502</v>
+      </c>
+      <c r="Z48">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="B49">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="C49" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D49">
-        <v>26.945203084574931</v>
+        <v>27.141428170684911</v>
       </c>
       <c r="E49">
-        <v>22.423372885417809</v>
+        <v>74.205514562532983</v>
       </c>
       <c r="F49">
-        <v>54.469166827601782</v>
+        <v>50.795139394736069</v>
       </c>
       <c r="G49">
-        <v>38.667004176022338</v>
+        <v>13.876890987594409</v>
       </c>
       <c r="H49">
-        <v>399.44864226640658</v>
+        <v>437.29671802253648</v>
       </c>
       <c r="I49">
-        <v>402.10594182481708</v>
+        <v>450.16820371038369</v>
       </c>
       <c r="J49">
-        <v>422.90907304513883</v>
+        <v>424.48849183203077</v>
       </c>
       <c r="K49">
-        <v>435.5821677117242</v>
+        <v>362.98327767688102</v>
       </c>
       <c r="L49">
-        <v>33.030887251015379</v>
+        <v>54.607081730162797</v>
       </c>
       <c r="M49">
-        <v>24.87777722703504</v>
+        <v>104.1460995556302</v>
       </c>
       <c r="N49">
-        <v>137.1861931594716</v>
+        <v>88.632730599537496</v>
       </c>
       <c r="O49">
-        <v>51.931955676615154</v>
-      </c>
-    </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.35">
+        <v>14.59337143572642</v>
+      </c>
+      <c r="X49">
+        <v>27.141428170684911</v>
+      </c>
+      <c r="Y49">
+        <v>54.607081730162797</v>
+      </c>
+      <c r="Z49">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="B50">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C50" t="s">
         <v>22</v>
       </c>
       <c r="D50">
-        <v>72.714689975159317</v>
+        <v>38.76855960345658</v>
       </c>
       <c r="E50">
-        <v>66.101522588720599</v>
+        <v>58.160357767798907</v>
       </c>
       <c r="F50">
-        <v>120.5457044660088</v>
+        <v>63.131696409314458</v>
       </c>
       <c r="G50">
-        <v>14.964361514912859</v>
+        <v>27.992737517673032</v>
       </c>
       <c r="H50">
-        <v>342.82560544463342</v>
+        <v>309.89218013465592</v>
       </c>
       <c r="I50">
-        <v>349.31096101940142</v>
+        <v>336.03554179181032</v>
       </c>
       <c r="J50">
-        <v>356.34237670949801</v>
+        <v>330.44036703039092</v>
       </c>
       <c r="K50">
-        <v>347.31626573204932</v>
+        <v>386.89860148852949</v>
       </c>
       <c r="L50">
-        <v>78.767348945561167</v>
+        <v>45.601378712452117</v>
       </c>
       <c r="M50">
-        <v>97.96779776425322</v>
+        <v>71.29228681988954</v>
       </c>
       <c r="N50">
-        <v>162.20144544955991</v>
+        <v>149.63878938188569</v>
       </c>
       <c r="O50">
-        <v>14.964361514912859</v>
-      </c>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.35">
+        <v>28.019281070537531</v>
+      </c>
+      <c r="X50">
+        <v>38.76855960345658</v>
+      </c>
+      <c r="Y50">
+        <v>45.601378712452117</v>
+      </c>
+      <c r="Z50">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="B51">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="C51" t="s">
         <v>22</v>
       </c>
       <c r="D51">
-        <v>105.206539158872</v>
+        <v>102.2273523737079</v>
       </c>
       <c r="E51">
-        <v>0</v>
+        <v>94.377073315763724</v>
       </c>
       <c r="F51">
-        <v>92.70002733563615</v>
+        <v>248.7240832590131</v>
       </c>
       <c r="G51">
-        <v>11.573012256991049</v>
+        <v>14.764428597060119</v>
       </c>
       <c r="H51">
-        <v>451.72797575651612</v>
+        <v>509.11392537154251</v>
       </c>
       <c r="I51">
-        <v>0</v>
+        <v>444.5394387903192</v>
       </c>
       <c r="J51">
-        <v>428.06619908093688</v>
+        <v>452.98134172715493</v>
       </c>
       <c r="K51">
-        <v>417.46739001997003</v>
+        <v>437.48115353530579</v>
       </c>
       <c r="L51">
-        <v>139.1265327313665</v>
+        <v>376.3303565989475</v>
       </c>
       <c r="M51">
-        <v>0</v>
+        <v>222.8020800528106</v>
       </c>
       <c r="N51">
-        <v>139.74694277204651</v>
+        <v>166.23762217502701</v>
       </c>
       <c r="O51">
-        <v>11.573012256991049</v>
-      </c>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.35">
+        <v>15.344741114274161</v>
+      </c>
+      <c r="X51">
+        <v>102.2273523737079</v>
+      </c>
+      <c r="Y51">
+        <v>376.3303565989475</v>
+      </c>
+      <c r="Z51">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="B52">
-        <v>12</v>
+        <v>111</v>
       </c>
       <c r="C52" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D52">
-        <v>109.73707886519161</v>
+        <v>39.531777047755639</v>
       </c>
       <c r="E52">
-        <v>261.13776919725211</v>
+        <v>68.82993429858297</v>
       </c>
       <c r="F52">
-        <v>226.34339234893409</v>
+        <v>78.35808245663813</v>
       </c>
       <c r="G52">
-        <v>11.605070703761021</v>
+        <v>88.061706532621713</v>
       </c>
       <c r="H52">
-        <v>489.83552856883159</v>
+        <v>328.38018664395059</v>
       </c>
       <c r="I52">
-        <v>261.13776919725211</v>
+        <v>304.35343389705952</v>
       </c>
       <c r="J52">
-        <v>496.22675882897698</v>
+        <v>323.05239826335497</v>
       </c>
       <c r="K52">
-        <v>505.79575177022258</v>
+        <v>425.28636284344708</v>
       </c>
       <c r="L52">
-        <v>189.9556814939302</v>
+        <v>103.178598349591</v>
       </c>
       <c r="M52">
-        <v>57.734343332197007</v>
+        <v>30.04465215964467</v>
       </c>
       <c r="N52">
-        <v>356.04000020375452</v>
+        <v>52.563559191054011</v>
       </c>
       <c r="O52">
-        <v>17.127483308572391</v>
-      </c>
-    </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.35">
+        <v>114.3666958345908</v>
+      </c>
+      <c r="X52">
+        <v>39.531777047755639</v>
+      </c>
+      <c r="Y52">
+        <v>103.178598349591</v>
+      </c>
+      <c r="Z52">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="B53">
-        <v>18</v>
+        <v>174</v>
       </c>
       <c r="C53" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D53">
-        <v>92.342254873128724</v>
-      </c>
-      <c r="E53">
-        <v>112.6809640903937</v>
+        <v>365.3432181055515</v>
       </c>
       <c r="F53">
-        <v>52.144533677607292</v>
+        <v>589.78607001776163</v>
       </c>
       <c r="G53">
-        <v>17.5963816071284</v>
+        <v>9.0162709181267644</v>
       </c>
       <c r="H53">
-        <v>320.04098190997871</v>
-      </c>
-      <c r="I53">
-        <v>338.44022593256699</v>
+        <v>620.04476798631129</v>
       </c>
       <c r="J53">
-        <v>355.71090011217842</v>
+        <v>623.47095650546771</v>
       </c>
       <c r="K53">
-        <v>371.69817777284209</v>
+        <v>398.00357604739531</v>
       </c>
       <c r="L53">
-        <v>99.709613853874075</v>
-      </c>
-      <c r="M53">
-        <v>120.190214958013</v>
+        <v>219.67073614440551</v>
       </c>
       <c r="N53">
-        <v>55.175647895780898</v>
+        <v>108.977655843035</v>
       </c>
       <c r="O53">
-        <v>19.168394322717209</v>
-      </c>
-    </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.35">
+        <v>11.44303999411494</v>
+      </c>
+      <c r="X53">
+        <v>365.3432181055515</v>
+      </c>
+      <c r="Y53">
+        <v>219.67073614440551</v>
+      </c>
+      <c r="Z53">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="B54">
-        <v>37</v>
+        <v>73</v>
       </c>
       <c r="C54" t="s">
         <v>22</v>
       </c>
       <c r="D54">
+        <v>49.727587386255557</v>
+      </c>
+      <c r="E54">
+        <v>95.758881643316855</v>
+      </c>
+      <c r="F54">
+        <v>91.643737142682156</v>
+      </c>
+      <c r="G54">
+        <v>32.109877716184577</v>
+      </c>
+      <c r="H54">
+        <v>404.99950839556197</v>
+      </c>
+      <c r="I54">
+        <v>407.03622005894118</v>
+      </c>
+      <c r="J54">
+        <v>384.84750083257723</v>
+      </c>
+      <c r="K54">
+        <v>473.64106558435049</v>
+      </c>
+      <c r="L54">
+        <v>105.7829253801773</v>
+      </c>
+      <c r="M54">
+        <v>214.14197337529961</v>
+      </c>
+      <c r="N54">
+        <v>175.71428013326999</v>
+      </c>
+      <c r="O54">
+        <v>37.910314583794097</v>
+      </c>
+      <c r="X54">
+        <v>49.727587386255557</v>
+      </c>
+      <c r="Y54">
+        <v>105.7829253801773</v>
+      </c>
+      <c r="Z54">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>62</v>
+      </c>
+      <c r="B55">
+        <v>27</v>
+      </c>
+      <c r="C55" t="s">
+        <v>22</v>
+      </c>
+      <c r="D55">
+        <v>23.646259520680751</v>
+      </c>
+      <c r="E55">
+        <v>23.301729159894919</v>
+      </c>
+      <c r="F55">
+        <v>32.020454442657062</v>
+      </c>
+      <c r="G55">
+        <v>29.24683532529318</v>
+      </c>
+      <c r="H55">
+        <v>412.25009682312958</v>
+      </c>
+      <c r="I55">
+        <v>403.94176964511178</v>
+      </c>
+      <c r="J55">
+        <v>384.67230012765248</v>
+      </c>
+      <c r="K55">
+        <v>381.49650965448711</v>
+      </c>
+      <c r="L55">
+        <v>24.738052884723761</v>
+      </c>
+      <c r="M55">
+        <v>23.89989208087173</v>
+      </c>
+      <c r="N55">
+        <v>38.701299967223129</v>
+      </c>
+      <c r="O55">
+        <v>29.761725902459961</v>
+      </c>
+      <c r="X55">
+        <v>23.646259520680751</v>
+      </c>
+      <c r="Y55">
+        <v>24.738052884723761</v>
+      </c>
+      <c r="Z55">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>65</v>
+      </c>
+      <c r="B56">
+        <v>15</v>
+      </c>
+      <c r="C56" t="s">
+        <v>22</v>
+      </c>
+      <c r="D56">
+        <v>72.714689975159317</v>
+      </c>
+      <c r="E56">
+        <v>66.101522588720599</v>
+      </c>
+      <c r="F56">
+        <v>120.5457044660088</v>
+      </c>
+      <c r="G56">
+        <v>14.964361514912859</v>
+      </c>
+      <c r="H56">
+        <v>342.82560544463342</v>
+      </c>
+      <c r="I56">
+        <v>349.31096101940142</v>
+      </c>
+      <c r="J56">
+        <v>356.34237670949801</v>
+      </c>
+      <c r="K56">
+        <v>347.31626573204932</v>
+      </c>
+      <c r="L56">
+        <v>78.767348945561167</v>
+      </c>
+      <c r="M56">
+        <v>97.96779776425322</v>
+      </c>
+      <c r="N56">
+        <v>162.20144544955991</v>
+      </c>
+      <c r="O56">
+        <v>14.964361514912859</v>
+      </c>
+      <c r="X56">
+        <v>72.714689975159317</v>
+      </c>
+      <c r="Y56">
+        <v>78.767348945561167</v>
+      </c>
+      <c r="Z56">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>66</v>
+      </c>
+      <c r="B57">
+        <v>9</v>
+      </c>
+      <c r="C57" t="s">
+        <v>22</v>
+      </c>
+      <c r="D57">
+        <v>105.206539158872</v>
+      </c>
+      <c r="F57">
+        <v>92.70002733563615</v>
+      </c>
+      <c r="G57">
+        <v>11.573012256991049</v>
+      </c>
+      <c r="H57">
+        <v>451.72797575651612</v>
+      </c>
+      <c r="J57">
+        <v>428.06619908093688</v>
+      </c>
+      <c r="K57">
+        <v>417.46739001997003</v>
+      </c>
+      <c r="L57">
+        <v>139.1265327313665</v>
+      </c>
+      <c r="N57">
+        <v>139.74694277204651</v>
+      </c>
+      <c r="O57">
+        <v>11.573012256991049</v>
+      </c>
+      <c r="X57">
+        <v>105.206539158872</v>
+      </c>
+      <c r="Y57">
+        <v>139.1265327313665</v>
+      </c>
+      <c r="Z57">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>69</v>
+      </c>
+      <c r="B58">
+        <v>37</v>
+      </c>
+      <c r="C58" t="s">
+        <v>22</v>
+      </c>
+      <c r="D58">
         <v>36.038054247813292</v>
       </c>
-      <c r="E54">
+      <c r="E58">
         <v>38.645026339439731</v>
       </c>
-      <c r="F54">
+      <c r="F58">
         <v>53.884552536286201</v>
       </c>
-      <c r="G54">
+      <c r="G58">
         <v>35.144824107681757</v>
       </c>
-      <c r="H54">
+      <c r="H58">
         <v>385.50033033582048</v>
       </c>
-      <c r="I54">
+      <c r="I58">
         <v>388.72324441609669</v>
       </c>
-      <c r="J54">
+      <c r="J58">
         <v>398.51141167916899</v>
       </c>
-      <c r="K54">
+      <c r="K58">
         <v>418.1757592887202</v>
       </c>
-      <c r="L54">
+      <c r="L58">
         <v>57.157642453515919</v>
       </c>
-      <c r="M54">
+      <c r="M58">
         <v>57.911536956388623</v>
       </c>
-      <c r="N54">
+      <c r="N58">
         <v>83.617921413370325</v>
       </c>
-      <c r="O54">
+      <c r="O58">
         <v>38.329765255636197</v>
       </c>
-    </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
-        <v>70</v>
-      </c>
-      <c r="B55">
-        <v>127</v>
-      </c>
-      <c r="C55" t="s">
-        <v>16</v>
-      </c>
-      <c r="D55">
-        <v>145.79226907872891</v>
-      </c>
-      <c r="E55">
-        <v>119.243151091578</v>
-      </c>
-      <c r="F55">
-        <v>227.21588577516371</v>
-      </c>
-      <c r="G55">
-        <v>18.594188650084359</v>
-      </c>
-      <c r="H55">
-        <v>416.81494970243853</v>
-      </c>
-      <c r="I55">
-        <v>398.62160931867243</v>
-      </c>
-      <c r="J55">
-        <v>405.1202850903386</v>
-      </c>
-      <c r="K55">
-        <v>423.23411992886292</v>
-      </c>
-      <c r="L55">
-        <v>44.02448729446192</v>
-      </c>
-      <c r="M55">
-        <v>49.661683396420337</v>
-      </c>
-      <c r="N55">
-        <v>36.532336388861793</v>
-      </c>
-      <c r="O55">
-        <v>21.252794080640541</v>
-      </c>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
-        <v>71</v>
-      </c>
-      <c r="B56">
-        <v>124</v>
-      </c>
-      <c r="C56" t="s">
-        <v>16</v>
-      </c>
-      <c r="D56">
-        <v>45.350272058957557</v>
-      </c>
-      <c r="E56">
-        <v>58.700289697901027</v>
-      </c>
-      <c r="F56">
-        <v>77.516673409048039</v>
-      </c>
-      <c r="G56">
-        <v>20.95128439121024</v>
-      </c>
-      <c r="H56">
-        <v>406.9102608456771</v>
-      </c>
-      <c r="I56">
-        <v>406.78224130167632</v>
-      </c>
-      <c r="J56">
-        <v>405.86090497093301</v>
-      </c>
-      <c r="K56">
-        <v>392.22590157363243</v>
-      </c>
-      <c r="L56">
-        <v>93.83477160384281</v>
-      </c>
-      <c r="M56">
-        <v>52.808598539760723</v>
-      </c>
-      <c r="N56">
-        <v>59.330492886414532</v>
-      </c>
-      <c r="O56">
-        <v>24.393175379022772</v>
-      </c>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
-        <v>72</v>
-      </c>
-      <c r="B57">
-        <v>49</v>
-      </c>
-      <c r="C57" t="s">
-        <v>16</v>
-      </c>
-      <c r="D57">
-        <v>53.222482281183758</v>
-      </c>
-      <c r="E57">
-        <v>63.298469519821687</v>
-      </c>
-      <c r="F57">
-        <v>65.863865836910421</v>
-      </c>
-      <c r="G57">
-        <v>12.90970715156589</v>
-      </c>
-      <c r="H57">
-        <v>376.16375212277097</v>
-      </c>
-      <c r="I57">
-        <v>368.43490525946271</v>
-      </c>
-      <c r="J57">
-        <v>378.11113342938671</v>
-      </c>
-      <c r="K57">
-        <v>381.35022296080172</v>
-      </c>
-      <c r="L57">
-        <v>69.126273897807906</v>
-      </c>
-      <c r="M57">
-        <v>114.8944866491285</v>
-      </c>
-      <c r="N57">
-        <v>137.98814458622681</v>
-      </c>
-      <c r="O57">
-        <v>13.40732613888288</v>
-      </c>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
-        <v>73</v>
-      </c>
-      <c r="B58">
-        <v>80</v>
-      </c>
-      <c r="C58" t="s">
-        <v>16</v>
-      </c>
-      <c r="D58">
-        <v>35.845989483527148</v>
-      </c>
-      <c r="E58">
-        <v>55.900912828113093</v>
-      </c>
-      <c r="F58">
-        <v>41.448538191005717</v>
-      </c>
-      <c r="G58">
-        <v>27.37782151530843</v>
-      </c>
-      <c r="H58">
-        <v>334.77724853747748</v>
-      </c>
-      <c r="I58">
-        <v>305.6194814065322</v>
-      </c>
-      <c r="J58">
-        <v>356.88648271383181</v>
-      </c>
-      <c r="K58">
-        <v>410.83967206156052</v>
-      </c>
-      <c r="L58">
-        <v>40.105904559271707</v>
-      </c>
-      <c r="M58">
-        <v>104.1427539838388</v>
-      </c>
-      <c r="N58">
-        <v>80.332767710706236</v>
-      </c>
-      <c r="O58">
-        <v>32.365358351714853</v>
-      </c>
-    </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="X58">
+        <v>36.038054247813292</v>
+      </c>
+      <c r="Y58">
+        <v>57.157642453515919</v>
+      </c>
+      <c r="Z58">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>74</v>
       </c>
@@ -3415,8 +4285,18 @@
       <c r="O59">
         <v>13.74741750028493</v>
       </c>
-    </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="X59">
+        <v>70.429943311341063</v>
+      </c>
+      <c r="Y59">
+        <v>99.301244211797666</v>
+      </c>
+      <c r="Z59">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>75</v>
       </c>
@@ -3462,8 +4342,18 @@
       <c r="O60">
         <v>32.101099371548891</v>
       </c>
-    </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="X60">
+        <v>23.93122205842781</v>
+      </c>
+      <c r="Y60">
+        <v>25.177471782345499</v>
+      </c>
+      <c r="Z60">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>76</v>
       </c>
@@ -3476,9 +4366,6 @@
       <c r="D61">
         <v>69.961910902257415</v>
       </c>
-      <c r="E61">
-        <v>0</v>
-      </c>
       <c r="F61">
         <v>299.36412438964811</v>
       </c>
@@ -3488,9 +4375,6 @@
       <c r="H61">
         <v>272.03784768399231</v>
       </c>
-      <c r="I61">
-        <v>0</v>
-      </c>
       <c r="J61">
         <v>469.13010252823392</v>
       </c>
@@ -3500,17 +4384,24 @@
       <c r="L61">
         <v>76.295936147590012</v>
       </c>
-      <c r="M61">
-        <v>0</v>
-      </c>
       <c r="N61">
         <v>161.87017436613499</v>
       </c>
       <c r="O61">
         <v>14.05666671150655</v>
       </c>
-    </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="X61">
+        <v>69.961910902257415</v>
+      </c>
+      <c r="Y61">
+        <v>76.295936147590012</v>
+      </c>
+      <c r="Z61">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>77</v>
       </c>
@@ -3556,8 +4447,18 @@
       <c r="O62">
         <v>31.681745261932399</v>
       </c>
-    </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="X62">
+        <v>80.087220384979702</v>
+      </c>
+      <c r="Y62">
+        <v>136.60300719840569</v>
+      </c>
+      <c r="Z62">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>78</v>
       </c>
@@ -3603,8 +4504,18 @@
       <c r="O63">
         <v>35.208806512833057</v>
       </c>
-    </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="X63">
+        <v>75.778988218410007</v>
+      </c>
+      <c r="Y63">
+        <v>110.6750525187782</v>
+      </c>
+      <c r="Z63">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>79</v>
       </c>
@@ -3650,8 +4561,18 @@
       <c r="O64">
         <v>44.300969100745561</v>
       </c>
-    </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="X64">
+        <v>63.788160401018743</v>
+      </c>
+      <c r="Y64">
+        <v>130.80796005139251</v>
+      </c>
+      <c r="Z64">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>80</v>
       </c>
@@ -3697,8 +4618,18 @@
       <c r="O65">
         <v>30.249860546764172</v>
       </c>
-    </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="X65">
+        <v>55.02203758361393</v>
+      </c>
+      <c r="Y65">
+        <v>78.218014481262301</v>
+      </c>
+      <c r="Z65">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>81</v>
       </c>
@@ -3744,8 +4675,18 @@
       <c r="O66">
         <v>23.839213054486489</v>
       </c>
-    </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="X66">
+        <v>48.176946718620258</v>
+      </c>
+      <c r="Y66">
+        <v>232.18956611066301</v>
+      </c>
+      <c r="Z66">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>82</v>
       </c>
@@ -3791,8 +4732,27 @@
       <c r="O67">
         <v>24.945667622185749</v>
       </c>
+      <c r="X67">
+        <v>57.79319035698061</v>
+      </c>
+      <c r="Y67">
+        <v>85.711345165422458</v>
+      </c>
+      <c r="Z67">
+        <f t="shared" ref="Z67" si="7">IF(X67&gt;Y67,1,0)</f>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:O67" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O67">
+      <sortCondition descending="1" ref="C1:C67"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="R4" formulaRange="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>